<commit_message>
UV check: the glass's lamp is 360-395 nm; 365 nm inspection, non-glowing banknote paper and optical brighteners cited from Mutanen et al. (IS&T PICS 2003), the ECB quick guide (2010) and US patent 6,918,482; paper added to the reference spreadsheet.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/literature/Review and paper links.xlsx
+++ b/docs/literature/Review and paper links.xlsx
@@ -3736,13 +3736,33 @@
       <c r="A61" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="13" t="n"/>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Luminescent Security Properties of Banknotes</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>https://www.imaging.org/common/uploaded%20files/pdfs/Papers/2003/PICS-0-287/8558.pdf</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
       <c r="E61" s="13" t="n"/>
-      <c r="F61" s="13" t="n"/>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>Conference Paper</t>
+        </is>
+      </c>
       <c r="G61" s="5" t="n"/>
-      <c r="H61" s="5" t="n"/>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>J. Mutanen, T. Jaaskelainen, J. P. S. Parkkinen (University of Joensuu). IS&amp;T's 2003 PICS Conference, pp. 421-424. Fluorescent fibres, inks and planchets in banknotes; the most widely used fluorescent security features are excited at 365 nm; banknote paper is non-fluorescent while most commercial papers contain whiteners that glow bluish under UV; a washed genuine note can glow too. Cited in the thesis (Literature review; UV fibre check).</t>
+        </is>
+      </c>
       <c r="I61" s="5" t="n"/>
       <c r="J61" s="5" t="n"/>
       <c r="K61" s="5" t="n"/>
@@ -31090,6 +31110,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>